<commit_message>
Gridsearch for loss implemented
</commit_message>
<xml_diff>
--- a/gridsearch_results_IMDB.xlsx
+++ b/gridsearch_results_IMDB.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +425,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LR</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>INNER_DIM</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>BATCH_SIZE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SOFTMAX_ASSIGN</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>DECREASE_PROPORTION</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_CONFIG_ID</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>VAL_MACRO_F1</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>COMPLETENESS</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>HYBRID_SCORE</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>MODEL_PATH</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_LINK</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_ENTROPY</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_RECONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_CONTRASTIVE</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_BALANCE</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>LOSS_REPEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="B2" t="n">
+        <v>64</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>all_large</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.7463</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.5402</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.6433</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>models/grid_search/IMDB/IMDB_DiffPool_20250602_163636_lr0.0001_hd100_bs16_softmaxTrue_dp0.1_lk1500.0_en0.2_rc0.1_ct0.01_bl0.1_rp0.1_f10.7463_comp0.5402_hyb0.6433_ep003.pth</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>